<commit_message>
Updated new generation of theory networks
</commit_message>
<xml_diff>
--- a/study_case_model/unit_networks/scenario_variables/demand_scenarios111.xlsx
+++ b/study_case_model/unit_networks/scenario_variables/demand_scenarios111.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>14362.67807379212</v>
+        <v>28095.85695202374</v>
       </c>
     </row>
     <row r="3">
@@ -482,7 +482,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -501,7 +501,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -509,6 +509,177 @@
         </is>
       </c>
       <c r="E4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>31165.45119995868</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>19612.9736849523</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>19</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Equinor Energy AS</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>23159.58912997847</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SHELL</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Vår Energi ASA</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>